<commit_message>
Publish pricing guide (no rates), owner-confirmed facts: statements-only patient billing, soften Ascend/bookkeeping/scope claims
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dental-refocus-url-status.xlsx
+++ b/docs/dental-refocus-url-status.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'URL status'!$A$1:$H$232</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'URL status'!$A$1:$H$239</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H232"/>
+  <dimension ref="A1:H239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -685,11 +685,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+          <t>https://rcm.texassolutions.co/blog/ai-in-dental-revenue-cycle-management/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>AI in Dental Revenue Cycle Management: What Automation Can and Cannot Do</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>301 -&gt; 200</t>
@@ -719,11 +727,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+          <t>https://rcm.texassolutions.co/blog/ai-in-dental-revenue-cycle-management/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>AI in Dental Revenue Cycle Management: What Automation Can and Cannot Do</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>301 -&gt; 200</t>
@@ -753,7 +769,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-billing-codes-guide/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-medical-cross-coding/</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -763,7 +779,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Dental Billing Codes Guide: How CDT Categories, Tooth Numbers and Surfaces Fit Together</t>
+          <t>Dental Medical Cross-Coding: Billing Medical Insurance for Dental Care</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1305,7 +1321,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Dental Billing Codes Guide: How CDT Categories, Tooth Numbers and Surfaces Fit Together</t>
+          <t>CDT Codes Explained: A Guide to Dental Codes, Tooth Numbers and Surfaces</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1337,11 +1353,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+          <t>https://rcm.texassolutions.co/blog/dental-insurance-biller/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>What Does a Dental Insurance Biller Do? Duties, Skills and Hiring Tips</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>301 -&gt; 200</t>
@@ -1895,11 +1919,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
+          <t>https://rcm.texassolutions.co/blog/ai-in-dental-revenue-cycle-management/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>AI in Dental Revenue Cycle Management: What Automation Can and Cannot Do</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
           <t>301 -&gt; 200</t>
@@ -1929,7 +1961,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-billing-codes-guide/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-medical-cross-coding/</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1939,7 +1971,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Dental Billing Codes Guide: How CDT Categories, Tooth Numbers and Surfaces Fit Together</t>
+          <t>Dental Medical Cross-Coding: Billing Medical Insurance for Dental Care</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2261,7 +2293,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>What Is Revenue Cycle Management for a Dental Practice?</t>
+          <t>What Is Dental Revenue Cycle Management (Dental RCM)?</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2847,7 +2879,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Dental Billing Services Across the United States</t>
+          <t>Dental Revenue Cycle Management Across the USA</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2885,7 +2917,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Dental Billing Services in California</t>
+          <t>Dental Revenue Cycle Management in California</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2923,7 +2955,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Dental Billing Services in Florida</t>
+          <t>Dental Revenue Cycle Management in Florida</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2961,7 +2993,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Dental Billing Services in New York</t>
+          <t>Dental Revenue Cycle Management in New York</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2999,7 +3031,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Dental Billing Services in Texas</t>
+          <t>Dental Revenue Cycle Management in Texas</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3895,17 +3927,17 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/services/dental-claims-processing/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-medical-cross-coding/</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Dental Claims Management</t>
+          <t>Dental Medical Cross-Coding: Billing Medical Insurance for Dental Care</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -8906,7 +8938,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/</t>
+          <t>https://rcm.texassolutions.co/blog/ada-dental-claim-form/</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -8922,12 +8954,12 @@
       <c r="D225" t="inlineStr"/>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Dental Carrier Billing and Claims Follow-Up</t>
+          <t>ADA Dental Claim Form: How to Fill It Out Correctly</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -8944,7 +8976,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/aetna/</t>
+          <t>https://rcm.texassolutions.co/blog/ai-in-dental-revenue-cycle-management/</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -8960,12 +8992,12 @@
       <c r="D226" t="inlineStr"/>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Aetna Dental Claims Billing &amp; Follow-Up</t>
+          <t>AI in Dental Revenue Cycle Management: What Automation Can and Cannot Do</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -8982,7 +9014,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/cigna/</t>
+          <t>https://rcm.texassolutions.co/blog/caqh-proview-for-dentists/</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -8998,12 +9030,12 @@
       <c r="D227" t="inlineStr"/>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Cigna Dental Claims Billing &amp; Follow-Up</t>
+          <t>ADA CAQH ProView for Dentists: Setup, Re-Attestation and Common Mistakes</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -9020,7 +9052,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/delta-dental/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-billing-software/</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -9036,12 +9068,12 @@
       <c r="D228" t="inlineStr"/>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Delta Dental Claims Billing &amp; Follow-Up</t>
+          <t>Dental Billing Software vs Outsourced Billing: What You Need</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -9058,7 +9090,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/guardian/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-insurance-biller/</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -9074,12 +9106,12 @@
       <c r="D229" t="inlineStr"/>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>Guardian Dental Claims Billing &amp; Follow-Up</t>
+          <t>What Does a Dental Insurance Biller Do? Duties, Skills and Hiring Tips</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -9096,7 +9128,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/metlife/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-medical-cross-coding/</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -9112,12 +9144,12 @@
       <c r="D230" t="inlineStr"/>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>MetLife Dental Claims Billing &amp; Follow-Up</t>
+          <t>Dental Medical Cross-Coding: Billing Medical Insurance for Dental Care</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -9134,7 +9166,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/unitedhealthcare-dental/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-practice-management-software/</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -9150,12 +9182,12 @@
       <c r="D231" t="inlineStr"/>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Dental Claims Billing &amp; Follow-Up</t>
+          <t>Dental Practice Management Software: How to Choose One</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -9172,7 +9204,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/pricing/</t>
+          <t>https://rcm.texassolutions.co/carriers/</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -9182,7 +9214,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Draft (not published)</t>
+          <t>New page</t>
         </is>
       </c>
       <c r="D232" t="inlineStr"/>
@@ -9193,12 +9225,12 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Dental Carrier Billing and Claims Follow-Up</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -9207,8 +9239,274 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/aetna/</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr"/>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Aetna Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/cigna/</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr"/>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Cigna Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/delta-dental/</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Delta Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/guardian/</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr"/>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Guardian Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/metlife/</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr"/>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>MetLife Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/unitedhealthcare-dental/</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr"/>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/pricing/</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr"/>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Dental RCM Pricing</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H232"/>
+  <autoFilter ref="A1:H239"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9219,7 +9517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -9250,40 +9548,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Draft (not published)</t>
+          <t>Kept (same URL)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kept (same URL)</t>
+          <t>New page</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>76</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>New page</t>
+          <t>Checks not OK</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Checks not OK</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Keyword gaps: 18 new posts (CDT codes, narratives, COB, UCR, KPIs...), page optimizations; remove all medical content (cross-coding post retired, HIPAA post renamed), only live calculator scripts built; trash button removes unused old terms
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dental-refocus-url-status.xlsx
+++ b/docs/dental-refocus-url-status.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'URL status'!$A$1:$H$239</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'URL status'!$A$1:$H$262</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +43,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000F1F3F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE68A"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,9 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H239"/>
+  <dimension ref="A1:H262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -769,7 +775,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-medical-cross-coding/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-billing-codes-guide/</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,7 +785,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Dental Medical Cross-Coding: Billing Medical Insurance for Dental Care</t>
+          <t>CDT Codes Explained: A Guide to Dental Codes, Tooth Numbers and Surfaces</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1428,10 +1434,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Kept (same URL)</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>301 redirect</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/hipaa-and-outsourced-dental-billing/</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>Blog post</t>
@@ -1444,7 +1454,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>301 -&gt; 200</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1961,7 +1971,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-medical-cross-coding/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-billing-codes-guide/</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1971,7 +1981,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Dental Medical Cross-Coding: Billing Medical Insurance for Dental Care</t>
+          <t>CDT Codes Explained: A Guide to Dental Codes, Tooth Numbers and Surfaces</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3572,10 +3582,14 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Kept (same URL)</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
+          <t>301 redirect</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/services/revenue-cycle-management/</t>
+        </is>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>Service</t>
@@ -3583,12 +3597,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Curve Dental Billing Services</t>
+          <t>Dental Revenue Cycle Management Services</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>301 -&gt; 200</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3927,7 +3941,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-medical-cross-coding/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-billing-codes-guide/</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -3937,7 +3951,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Dental Medical Cross-Coding: Billing Medical Insurance for Dental Care</t>
+          <t>CDT Codes Explained: A Guide to Dental Codes, Tooth Numbers and Surfaces</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -7793,7 +7807,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Dental Insurance Verification Checklist</t>
+          <t>Dental Insurance Verification Form and Checklist</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -7979,7 +7993,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Fee Schedule Comparison Calculator</t>
+          <t>Dental Fee Schedule Comparison Calculator</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -9052,7 +9066,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-billing-software/</t>
+          <t>https://rcm.texassolutions.co/blog/d4346-vs-d1110/</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -9073,7 +9087,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Dental Billing Software vs Outsourced Billing: What You Need</t>
+          <t>D4346 vs D1110: Gingivitis Scaling or Prophylaxis?</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -9090,7 +9104,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-insurance-biller/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-billing-software/</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -9111,7 +9125,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>What Does a Dental Insurance Biller Do? Duties, Skills and Hiring Tips</t>
+          <t>Dental Billing Software vs Outsourced Billing: What You Need</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -9128,7 +9142,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-medical-cross-coding/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-carc-rarc-denial-codes/</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -9149,7 +9163,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Dental Medical Cross-Coding: Billing Medical Insurance for Dental Care</t>
+          <t>CARC Codes and RARC Codes on Dental Claims: How to Read and Act on Them</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -9166,7 +9180,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/blog/dental-practice-management-software/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-coordination-of-benefits/</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -9187,7 +9201,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Dental Practice Management Software: How to Choose One</t>
+          <t>Dental Coordination of Benefits: Primary, Secondary and COB Rules</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -9204,7 +9218,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-crown-codes/</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -9220,12 +9234,12 @@
       <c r="D232" t="inlineStr"/>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Dental Carrier Billing and Claims Follow-Up</t>
+          <t>Dental Crown Codes: D2740, D2950 and Seat Date Billing</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -9242,7 +9256,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/aetna/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-exam-codes-d0120-d0140-d0150/</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -9258,12 +9272,12 @@
       <c r="D233" t="inlineStr"/>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Aetna Dental Claims Billing &amp; Follow-Up</t>
+          <t>Dental Exam Codes: D0120, D0140 and D0150 Explained</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -9280,7 +9294,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/cigna/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-extraction-codes-d7140-d7210/</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -9296,12 +9310,12 @@
       <c r="D234" t="inlineStr"/>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Cigna Dental Claims Billing &amp; Follow-Up</t>
+          <t>Dental Extraction Codes: D7140 vs D7210 for Billing</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -9318,7 +9332,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/delta-dental/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-front-desk-insurance-checklist/</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -9334,12 +9348,12 @@
       <c r="D235" t="inlineStr"/>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Delta Dental Claims Billing &amp; Follow-Up</t>
+          <t>Dental Front Desk Insurance Checklist: Daily and Weekly Tasks</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -9356,7 +9370,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/guardian/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-implant-codes/</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -9372,12 +9386,12 @@
       <c r="D236" t="inlineStr"/>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Guardian Dental Claims Billing &amp; Follow-Up</t>
+          <t>Dental Implant Codes: A Billing Guide to D6010, D6011 and Implant Crowns</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -9394,7 +9408,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/metlife/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-insurance-biller/</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -9410,12 +9424,12 @@
       <c r="D237" t="inlineStr"/>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>MetLife Dental Claims Billing &amp; Follow-Up</t>
+          <t>What Does a Dental Insurance Biller Do? Duties, Skills and Hiring Tips</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -9432,7 +9446,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/carriers/unitedhealthcare-dental/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-insurance-narratives/</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -9448,12 +9462,12 @@
       <c r="D238" t="inlineStr"/>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Blog post</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Dental Claims Billing &amp; Follow-Up</t>
+          <t>Dental Narratives: How to Write Them, With Sample Templates</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -9470,7 +9484,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>https://rcm.texassolutions.co/pricing/</t>
+          <t>https://rcm.texassolutions.co/blog/dental-office-manager-billing-duties/</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -9486,27 +9500,901 @@
       <c r="D239" t="inlineStr"/>
       <c r="E239" t="inlineStr">
         <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Dental Office Manager and Treatment Coordinator Roles in the Revenue Cycle</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/dental-practice-kpis/</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr"/>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Dental KPIs: The Revenue Cycle Numbers Every Practice Should Track</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/dental-practice-management-software/</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr"/>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Dental Practice Management Software: How to Choose One</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/dental-predetermination-vs-preauthorization/</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr"/>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Dental Predetermination vs Pre-Authorization: What Is the Difference?</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/dental-x-ray-codes/</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr"/>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Dental X-Ray Codes: Bitewings, D0220, D0210 and Pano</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/dhmo-vs-ppo-for-dental-practices/</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr"/>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Dental PPO vs HMO: What Each Plan Type Means for Your Practice</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/hipaa-and-outsourced-dental-billing/</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr"/>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>HIPAA and Outsourced Dental Billing: What Practices Should Know</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/in-house-dental-membership-plans/</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr"/>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>In-House Dental Membership Plans: How They Work and What to Check</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/missing-tooth-clause/</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr"/>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Missing Tooth Clause: What It Is and How Dental Offices Handle It</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/periodontal-codes-d4341-d4342-d4910-d4355/</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr"/>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>D4341 vs D4342, D4910 and D4355: A Billing Guide to Periodontal Codes</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/blog/ucr-fees-dental/</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr"/>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Blog post</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Dental UCR Fees: What UCR Means and How It Affects Your Fee Schedule</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr"/>
+      <c r="E250" t="inlineStr">
+        <is>
           <t>Page</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr">
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Dental Carrier Billing and Claims Follow-Up</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/aetna/</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr"/>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Aetna Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/cigna/</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr"/>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Cigna Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/delta-dental/</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr"/>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Delta Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/guardian/</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr"/>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Guardian Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/metlife/</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr"/>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>MetLife Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/carriers/unitedhealthcare-dental/</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr"/>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Dental Claims Billing &amp; Follow-Up</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/pricing/</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr"/>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
         <is>
           <t>Dental RCM Pricing</t>
         </is>
       </c>
-      <c r="G239" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="H239" t="inlineStr">
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/tools/dental-annual-maximum-calculator/</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr"/>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Dental Annual Maximum Calculator</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/tools/dental-credentialing-revenue-calculator/</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr"/>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Dental Credentialing Revenue Calculator</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/tools/dental-denial-cost-calculator/</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr"/>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Dental Claim Denial Cost Calculator</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/tools/dental-patient-estimate-calculator/</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr"/>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Dental Insurance Estimate Calculator</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>https://rcm.texassolutions.co/tools/dental-ppo-write-off-calculator/</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>New page</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr"/>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Dental PPO Write-Off Calculator</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H239"/>
+  <autoFilter ref="A1:H262"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9542,7 +10430,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3">
@@ -9552,7 +10440,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
@@ -9562,7 +10450,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -9572,7 +10460,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh URL status report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dental-refocus-url-status.xlsx
+++ b/docs/dental-refocus-url-status.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -43,11 +43,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000F1F3F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDE68A"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,10 +58,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9586,12 +9580,12 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H241" s="2" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -10460,7 +10454,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>